<commit_message>
Add multilingual translation and voice features
</commit_message>
<xml_diff>
--- a/backend/Scholarship_Verification.xlsx
+++ b/backend/Scholarship_Verification.xlsx
@@ -435,12 +435,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
@@ -450,9 +450,9 @@
     <col width="45" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="45" customWidth="1" min="14" max="14"/>
-    <col width="23" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
     <col width="22" customWidth="1" min="16" max="16"/>
     <col width="25" customWidth="1" min="17" max="17"/>
   </cols>
@@ -726,12 +726,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>₹80,000/yr + ₹20,000 mentorship</t>
+          <t>Rs. 80,000/yr + Rs. 20,000 mentorship</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>₹5</t>
+          <t>Rs. 80,000/yr + Rs. 20,000 mentorship</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>31 December 2026</t>
+          <t>Rolling (renewal every year)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Subsumed / Merged (INSPIRE)</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -791,17 +791,17 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>REQUIREMENT MISMATCH</t>
+          <t>VERIFIED ELIGIBLE</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 20:50:06</t>
+          <t>2026-08-31 13:15:37</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>DO NOT RECOMMEND</t>
+          <t>RECOMMEND</t>
         </is>
       </c>
     </row>
@@ -813,12 +813,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Up to ₹1,00,000+</t>
+          <t>Up to Rs. 1,00,000+</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Up to ₹1,00,000+</t>
+          <t>Up to Rs. 1,00,000+</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -868,12 +868,12 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>buildyourfuture.withgoogle.com</t>
+          <t>https://scholarships.gov.in</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 21:18:35</t>
+          <t>2026-08-31 12:07:31</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 14:01:16</t>
+          <t>2026-08-30 17:39:29</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
@@ -1144,10 +1144,532 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 14:17:46</t>
+          <t>2026-08-31 13:14:44</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Narotam Sekhsaria Foundation Scholarship</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Up to Rs. 6,00,000 (loan-scholarship)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Up to Rs. 6,00,000 (loan-scholarship)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Combination of scholarship + soft loan for masters study</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: Strong academic record + financial need, ₹600,000</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Strong academic record + financial need</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Strong academic record + financial need</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>₹600,000</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>₹600,000</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Mar - May</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Mar - May</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>https://pg.nsfoundation.co.in/programme/</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-30 17:39:28</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Reliance Foundation Undergraduate Scholarship</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Up to Rs. 2,00,000 (over degree)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>₹2</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Selection via online aptitude test; includes mentorship</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: Merit + aptitude test, Not Found</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Merit + aptitude test</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Merit + aptitude test</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Aug - Oct</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Aug - Oct</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>https://articles.findmycollege.com/reliance-foundation-scholarships-details/</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31 11:51:54</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>PM-USP Central Sector Scheme (PM Scholarship)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 82,000/yr (approx.)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 82,000/yr (approx.)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Formerly known as CSS; income limit is stricter subtype</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: 80, ≤ ₹450,000</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>80th percentile Class 12</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>₹450,000</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>≤ ₹450,000</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>https://scholarships.gov.in</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31 12:13:15</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Central Sector Scholarship for College &amp; University Students (ex-CSSS renewal)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 10,000 - Rs. 20,000/yr</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 10,000 - Rs. 20,000/yr</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Renewal application track of CSSS</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: Maintain 50%+ each year, ≤ ₹800,000</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Maintain 50%+ each year</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Maintain 50%+ each year</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>₹800,000</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>≤ ₹800,000</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>https://scholarships.gov.in</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31 12:56:35</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>IDFC FIRST Bank Scholarship</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Varies (tuition support)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Varies (tuition support)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>CSR-driven scheme for meritorious low-income students</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: Merit-cum-means, ₹250,000</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Merit-cum-means</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Merit-cum-means</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>₹250,000</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>₹250,000</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Varies</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Varies</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.idfcfirst.bank.in/csr-activities/educational-initiatives/mba-scholarship</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31 12:59:35</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Pudhumai Penn Scheme</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 1,000/month till graduation</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 1,000/month till graduation</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Direct benefit transfer scheme for girl students</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: Studied Class 6 - 12 in Govt/Aided Tamil-medium school, Not Found</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Studied Class 6 - 12 in Govt/Aided Tamil-medium school</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Studied Class 6 - 12 in Govt/Aided Tamil-medium school</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Automatic on admission (verify with college)</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Automatic on admission (verify with college)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.myscheme.gov.in/schemes/pudhumai-penn-scheme</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31 13:03:06</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
         <is>
           <t>RECOMMEND</t>
         </is>

</xml_diff>

<commit_message>
Add latest project updates
</commit_message>
<xml_diff>
--- a/backend/Scholarship_Verification.xlsx
+++ b/backend/Scholarship_Verification.xlsx
@@ -915,7 +915,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Active online with criteria: Merit-based, Not Found</t>
+          <t>Active online with criteria: 2.25, Not Found</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Merit-based</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 17:39:29</t>
+          <t>2026-09-05 23:01:06</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 17:39:28</t>
+          <t>2026-09-01 13:53:28</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>https://articles.findmycollege.com/reliance-foundation-scholarships-details/</t>
+          <t>https://dasmail.reliancefoundation.org/UG_Scholarship.aspx</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 11:51:54</t>
+          <t>2026-09-05 22:42:01</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update latest project changes
</commit_message>
<xml_diff>
--- a/backend/Scholarship_Verification.xlsx
+++ b/backend/Scholarship_Verification.xlsx
@@ -435,12 +435,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
@@ -905,7 +905,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>₹50,000</t>
+          <t>Rs. 50,000 (1-time)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/reel/DFJ4O2sy2uT/</t>
+          <t>https://unstop.com/scholarships/virtusa-engineering-excellence-scholarship-2024-25-virtusa-1359876</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 23:01:06</t>
+          <t>2026-09-25 16:08:54</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>https://pg.nsfoundation.co.in/programme/</t>
+          <t>https://www.studentcover.in/narotam-sekhsaria-scholarship/</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 13:53:28</t>
+          <t>2026-09-21 10:04:01</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>₹2</t>
+          <t>₹2 lakh</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>https://dasmail.reliancefoundation.org/UG_Scholarship.aspx</t>
+          <t>https://www.scholarships.reliancefoundation.org/assets/pdf/PG_FAQ.pdf</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 22:42:01</t>
+          <t>2026-09-25 13:33:31</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
@@ -1670,6 +1670,354 @@
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Top Class Education Scheme for SC Students</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Full tuition + maintenance (up to Rs. 2,00,000)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Full tuition + maintenance (up to Rs. 2,00,000)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Only for admissions into notified top institutes (IITs, IIMs, NITs etc.)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: Merit-based admission, ₹800,000</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Merit-based admission</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Merit-based admission</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>₹800,000</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>₹800,000</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/goimsje/posts/the-top-class-education-scholarship-supports-sc-students-in-pursuing-higher-educ/1443282421315987/</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:07:03</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Aditya Birla Scholarship</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Up to Rs. 1,75,000/yr</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>₹,</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Restricted to specific premier institutes</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: Top academic rank at partner institute, Not Found</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Top academic rank at partner institute</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Top academic rank at partner institute</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Aug - Sep</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Aug - Sep</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adityabirlascholars.net/the-scholarship/</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 09:21:04</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>JN Tata Endowment Loan Scholarship</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 1,00,000 - Rs. 10,00,000 (loan scholarship)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>₹20 lakh</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Interest-free loan-scholarship for postgraduate studies</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: Strong academic record, Not Found</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Strong academic record</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Strong academic record</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Feb - Apr</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Feb - Apr</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>https://application.jntataendowment.org/TataEndowment/</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 12:37:21</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Merit-cum-Means Scholarship for Minorities (Technical/Professional)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Tuition (up to Rs. 20,000) + Rs. 1,000 - 1,200/month</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Tuition (up to Rs. 20,000) + Rs. 1,000 - 1,200/month</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>For professional &amp; technical courses only</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: 50%, ≤ ₹250,000</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>50% in prev. exam</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>₹250,000</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>≤ ₹250,000</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>https://scholarships.gov.in</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:01:45</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
         <is>
           <t>RECOMMEND</t>
         </is>

</xml_diff>

<commit_message>
Update scholarship verification and workflow
</commit_message>
<xml_diff>
--- a/backend/Scholarship_Verification.xlsx
+++ b/backend/Scholarship_Verification.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 12:56:35</t>
+          <t>2026-09-25 21:05:20</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
@@ -2101,12 +2101,99 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 19:38:10</t>
+          <t>2026-09-25 19:47:10</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
           <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Sitaram Jindal Foundation Scholarship</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Up to Rs. 24,000/yr</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>₹4000</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Renewable annually with academic progress</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: Merit-cum-means, ≤ ₹2</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Merit-cum-means</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Merit-cum-means</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>₹250,000</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>≤ ₹2</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Jul - Sep</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Jul - Sep</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>https://theglobalscholarship.org/scholarships/sitaram-jindal-foundation-scholarship-2025?source=main</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>NOT ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 21:08:02</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>DO NOT RECOMMEND</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ocr): correct V to Y confusion in extracted names and sanitize against student profile
</commit_message>
<xml_diff>
--- a/backend/Scholarship_Verification.xlsx
+++ b/backend/Scholarship_Verification.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Logs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Verification Logs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -2197,6 +2197,93 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>National Means-cum-Merit Scholarship (NMMS)</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 12,000/yr (Rs. 1,000/month)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 12,000/yr (Rs. 1,000/month)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Selection via state-level MAT+SAT exam at Class 8</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: 55% in Class 7 (Class 8 selection test), ≤ ₹3</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>55% in Class 7 (Class 8 selection test)</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>55% in Class 7 (Class 8 selection test)</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>₹350,000</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>≤ ₹3</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct (state-wise varies)</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct (state-wise varies)</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>https://rajshaladarpan.rajasthan.gov.in/sd1/NMMS/Home.aspx</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED ELIGIBLE</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 07:09:23</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: Resolve case-sensitive document matching in scholarship journey widget
</commit_message>
<xml_diff>
--- a/backend/Scholarship_Verification.xlsx
+++ b/backend/Scholarship_Verification.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -2284,6 +2284,93 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Swayam Charitable Trust Aspire Scholarship</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Varies (tuition support)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Varies (tuition support)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Founded by HCL co-founder Dr. Ajai Chowdhry</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Active online with criteria: Merit + financial need, ₹300,000</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Merit + financial need</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Merit + financial need</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>₹300,000</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>₹300,000</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Varies</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Varies</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.co.in/intl/en/about/products?tab=wh</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>PARTIALLY VERIFIED</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 09:09:46</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMEND</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Feat: Target 2026 academic year in RPA verification queries and deduplicate criteria
</commit_message>
<xml_diff>
--- a/backend/Scholarship_Verification.xlsx
+++ b/backend/Scholarship_Verification.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Verification Logs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Logs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -552,52 +552,52 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>₹10,000/yr (UG), ₹20,000/yr (PG)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>₹8</t>
+          <t>₹,</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>Apply fresh + renewal every year on NSP</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Active online with criteria: Not Available, Not Available</t>
+          <t>Active online with criteria: Top 20th percentile in Class 12, ≤ ₹4</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>Top 20th percentile in Class 12</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>Top 20th percentile in Class 12</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>₹800,000</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>≤ ₹4</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>31 Oct</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>31 October 2026</t>
+          <t>31 Oct</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>https://motion.ac.in/examinfo/cbse-scholarship/</t>
+          <t>https://scholarships.gov.in/</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 19:04:07</t>
+          <t>2026-09-26 09:34:53</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
@@ -813,32 +813,28 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Up to Rs. 1,00,000+</t>
+          <t>Not Available</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Up to Rs. 1,00,000+</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Application via Google's scholarship portal; competitive selection</t>
-        </is>
-      </c>
+          <t>Standard grant as per norms</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Active online with criteria: Strong CS academic background, Not Found</t>
+          <t>Active online with criteria: Not Found, Not Found</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Strong CS academic background</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Strong CS academic background</t>
+          <t>Not Found</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -853,12 +849,12 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Varies (usually mid-year)</t>
+          <t>31-03-2026</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Varies (usually mid-year)</t>
+          <t>31-03-2026</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -878,17 +874,17 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>NOT ELIGIBLE</t>
+          <t>VERIFIED ELIGIBLE</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 12:07:31</t>
+          <t>2026-09-26 09:37:55</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>DO NOT RECOMMEND</t>
+          <t>RECOMMEND</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1075,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Rs. 75,000 - Rs. 1,25,000/yr</t>
+          <t>₹1,25,000 annual</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1089,7 +1085,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Active online with criteria: Merit via entrance exam, ≤ ₹250,000</t>
+          <t>Active online with criteria: Merit via entrance exam, ₹250,000</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1109,7 +1105,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>≤ ₹250,000</t>
+          <t>₹250,000</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1134,7 +1130,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>https://scholarships.gov.in</t>
+          <t>https://www.indiascholarships.in/scholarships/pm-yasasvi-top-class-education</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1144,7 +1140,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 13:14:44</t>
+          <t>2026-09-26 09:31:53</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">

</xml_diff>